<commit_message>
dates made consistently in day-month-year order
</commit_message>
<xml_diff>
--- a/data/aura_motion_visualization.xlsx
+++ b/data/aura_motion_visualization.xlsx
@@ -569,12 +569,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>5-Jun-2024</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>5 Jun 2024</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>June 5, 2024</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -621,17 +621,17 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>February 5, 2024</t>
+          <t>5.2.2024</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>28-Mar-2024</t>
+          <t>28-3-2024</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Mar 28, 2024</t>
+          <t>28 Mar, 2024</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>September 17, 2024</t>
+          <t>17-Sep-2024</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -727,17 +727,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>16-Jan-2024</t>
+          <t>16.1.2024</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>28-2-2024</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>February 28, 2024</t>
+          <t>28 Feb, 2024</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -784,17 +784,17 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Jun 6, 2024</t>
+          <t>6/6/2024</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>28/7/2024</t>
+          <t>28-Jul-2024</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>July 28, 2024</t>
+          <t>28 Jul 2024</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -841,12 +841,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>8 Mar 2024</t>
+          <t>8.3.2024</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>28-Mar-2024</t>
+          <t>28-3-2024</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr"/>
@@ -894,17 +894,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>5 Jun 2024</t>
+          <t>5 Jun, 2024</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Jul 19, 2024</t>
+          <t>19/7/2024</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>19/7/2024</t>
+          <t>19-Jul-2024</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -951,12 +951,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>September 24, 2024</t>
+          <t>24 Sep 2024</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>28-Sep-2024</t>
+          <t>28.9.2024</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr"/>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>May 13, 2024</t>
+          <t>13-5-2024</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>25/6/2024</t>
+          <t>25 Jun, 2024</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>June 28, 2024</t>
+          <t>28/6/2024</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1066,12 +1066,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Mar 28, 2024</t>
+          <t>28 Mar 2024</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>March 28, 2024</t>
+          <t>28.3.2024</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1118,17 +1118,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>May 4, 2024</t>
+          <t>4-5-2024</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
+          <t>22 Jun, 2024</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
           <t>22/6/2024</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>June 22, 2024</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1175,17 +1175,17 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>10 Apr 2024</t>
+          <t>10-Apr-2024</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>26/05/2024</t>
+          <t>26 May 2024</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>28 May 2024</t>
+          <t>28.5.2024</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1232,12 +1232,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>9-Mar-2024</t>
+          <t>9-3-2024</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Apr 23, 2024</t>
+          <t>23 Apr, 2024</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>May 16, 2024</t>
+          <t>16-May-2024</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>18/07/2024</t>
+          <t>18 Jul 2024</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>23-Jul-2024</t>
+          <t>23.7.2024</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1342,17 +1342,17 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>20 Aug 2024</t>
+          <t>20-8-2024</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>28/09/2024</t>
+          <t>28 Sep, 2024</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Sep 28, 2024</t>
+          <t>28/9/2024</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1399,17 +1399,17 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>August 2, 2024</t>
+          <t>2-Aug-2024</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>28/9/2024</t>
+          <t>28 Sep 2024</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>September 28, 2024</t>
+          <t>28.9.2024</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1452,12 +1452,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>3-Mar-2024</t>
+          <t>3-3-2024</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>May 6, 2024</t>
+          <t>6 May, 2024</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1505,17 +1505,17 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>August 13, 2024</t>
+          <t>13-Aug-2024</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>September 20, 2024</t>
+          <t>20 Sep 2024</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>25/09/2024</t>
+          <t>25.9.2024</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2-Aug-2024</t>
+          <t>2-8-2024</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>October 6, 2024</t>
+          <t>6 Oct, 2024</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1619,12 +1619,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>19/07/2024</t>
+          <t>19-Jul-2024</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Jul 28, 2024</t>
+          <t>28 Jul 2024</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr"/>
@@ -1672,17 +1672,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>August 7, 2024</t>
+          <t>7.8.2024</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>September 28, 2024</t>
+          <t>28-9-2024</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>September 28, 2024</t>
+          <t>28 Sep, 2024</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>17 Jun 2024</t>
+          <t>17/6/2024</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>17/07/2024</t>
+          <t>17-Jul-2024</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1786,17 +1786,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>June 21, 2024</t>
+          <t>21.6.2024</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>28/6/2024</t>
+          <t>28-6-2024</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>28 Jun 2024</t>
+          <t>28 Jun, 2024</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1843,12 +1843,12 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>June 21, 2024</t>
+          <t>21/6/2024</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>June 28, 2024</t>
+          <t>28-Jun-2024</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1900,17 +1900,17 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>10/09/2024</t>
+          <t>10.9.2024</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>28/09/2024</t>
+          <t>28-9-2024</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>28/09/2024</t>
+          <t>28 Sep, 2024</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1957,12 +1957,12 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>9-Oct-2024</t>
+          <t>9/10/2024</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Nov 28, 2024</t>
+          <t>28-Nov-2024</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -2010,17 +2010,17 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>5/10/2024</t>
+          <t>5.10.2024</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>November 11, 2024</t>
+          <t>11-11-2024</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>28/11/2024</t>
+          <t>28 Nov, 2024</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2067,12 +2067,12 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>7 Jun 2024</t>
+          <t>7/6/2024</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>28/06/2024</t>
+          <t>28-Jun-2024</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -2124,17 +2124,17 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>05/07/2024</t>
+          <t>5.7.2024</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>7-Aug-2024</t>
+          <t>7-8-2024</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Aug 28, 2024</t>
+          <t>28 Aug, 2024</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>27 Jul 2024</t>
+          <t>27-Jul-2024</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>July 28, 2024</t>
+          <t>28 Jul 2024</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2238,17 +2238,17 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>September 18, 2024</t>
+          <t>18.9.2024</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>28 Oct 2024</t>
+          <t>28-10-2024</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>28-Oct-2024</t>
+          <t>28 Oct, 2024</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2295,17 +2295,17 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Jul 5, 2024</t>
+          <t>5/7/2024</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>6/9/2024</t>
+          <t>6-Sep-2024</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>September 16, 2024</t>
+          <t>16 Sep 2024</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2348,17 +2348,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>18-Aug-2024</t>
+          <t>18.8.2024</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Sep 25, 2024</t>
+          <t>25-9-2024</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>25/9/2024</t>
+          <t>25 Sep, 2024</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2405,17 +2405,17 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>September 13, 2024</t>
+          <t>13/9/2024</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>24 Oct 2024</t>
+          <t>24-Oct-2024</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>October 28, 2024</t>
+          <t>28 Oct 2024</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2462,17 +2462,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>January 22, 2024</t>
+          <t>22.1.2024</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>28-2-2024</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>28 Feb, 2024</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2519,17 +2519,17 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>21-Feb-2024</t>
+          <t>21/2/2024</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Mar 28, 2024</t>
+          <t>28-Mar-2024</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>28/3/2024</t>
+          <t>28 Mar 2024</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2576,17 +2576,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>August 9, 2024</t>
+          <t>9.8.2024</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>28-Aug-2024</t>
+          <t>28-8-2024</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>28/08/2024</t>
+          <t>28 Aug, 2024</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2633,12 +2633,12 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Apr 1, 2024</t>
+          <t>1/4/2024</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>3/5/2024</t>
+          <t>3-May-2024</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr"/>
@@ -2686,17 +2686,17 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>05/04/2024</t>
+          <t>5 Apr 2024</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>21 May 2024</t>
+          <t>21.5.2024</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>May 26, 2024</t>
+          <t>26-5-2024</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2743,17 +2743,17 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>September 17, 2024</t>
+          <t>17 Sep, 2024</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
+          <t>28/9/2024</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
           <t>28-Sep-2024</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>September 28, 2024</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2800,17 +2800,17 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Jul 9, 2024</t>
+          <t>9 Jul 2024</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>23/7/2024</t>
+          <t>23.7.2024</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>28/07/2024</t>
+          <t>28-7-2024</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2857,12 +2857,12 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>July 13, 2024</t>
+          <t>13 Jul, 2024</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>28-Jul-2024</t>
+          <t>28/7/2024</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr"/>
@@ -2910,17 +2910,17 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>07/05/2024</t>
+          <t>7-May-2024</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Jul 11, 2024</t>
+          <t>11 Jul 2024</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>11/07/2024</t>
+          <t>11.7.2024</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2967,12 +2967,12 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>May 8, 2024</t>
+          <t>8-5-2024</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>July 12, 2024</t>
+          <t>12 Jul, 2024</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -3024,17 +3024,17 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>August 2, 2024</t>
+          <t>2-Aug-2024</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>10-Sep-2024</t>
+          <t>10 Sep 2024</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>28 Sep 2024</t>
+          <t>28.9.2024</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3081,17 +3081,17 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>February 15, 2024</t>
+          <t>15-2-2024</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>24/03/2024</t>
+          <t>24 Mar, 2024</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>24/03/2024</t>
+          <t>24/3/2024</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3134,17 +3134,17 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Aug 8, 2024</t>
+          <t>8-Aug-2024</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>10/10/2024</t>
+          <t>10 Oct 2024</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>October 5, 2024</t>
+          <t>5.10.2024</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3191,12 +3191,12 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>8-Oct-2024</t>
+          <t>8-10-2024</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>Oct 28, 2024</t>
+          <t>28 Oct, 2024</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>06/06/2024</t>
+          <t>6-Jun-2024</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -3297,17 +3297,17 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>16 Oct 2024</t>
+          <t>16.10.2024</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>December 16, 2024</t>
+          <t>16-12-2024</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>December 16, 2024</t>
+          <t>16 Dec, 2024</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
@@ -3354,17 +3354,17 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>13-May-2024</t>
+          <t>13/5/2024</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>May 28, 2024</t>
+          <t>28-May-2024</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>28/5/2024</t>
+          <t>28 May 2024</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -3411,17 +3411,17 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>June 19, 2024</t>
+          <t>19.6.2024</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>June 28, 2024</t>
+          <t>28-6-2024</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>28 Jun 2024</t>
+          <t>28 Jun, 2024</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
@@ -3460,17 +3460,17 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>6-May-2024</t>
+          <t>6/5/2024</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Jun 28, 2024</t>
+          <t>28-Jun-2024</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>June 28, 2024</t>
+          <t>28 Jun 2024</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -3517,17 +3517,17 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>18/6/2024</t>
+          <t>18.6.2024</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>July 28, 2024</t>
+          <t>28-7-2024</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>28-Jul-2024</t>
+          <t>28 Jul, 2024</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -3574,12 +3574,12 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Feb 5, 2024</t>
+          <t>5/2/2024</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>24 Feb 2024</t>
+          <t>24-Feb-2024</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr"/>
@@ -3627,17 +3627,17 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>6/7/2024</t>
+          <t>6 Jul 2024</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>July 28, 2024</t>
+          <t>28.7.2024</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>28-Jul-2024</t>
+          <t>28-7-2024</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">

</xml_diff>